<commit_message>
Fix PER calculation and add IFRS/negative-number handling to Excel export
FEPS/FDivAnn now only read from FY-tagged disclosures, avoiding a
quarterly forecast-revision row being misread as a full-year forecast
(caused PER to be wildly inflated). Also fall back to operating profit
for ordinary-profit rows when a company reports under IFRS (no
ordinary-profit concept), and switch negative-number display from
parentheses to ▲ across both templates.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/company_detail_template.xlsx
+++ b/templates/company_detail_template.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17325" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="原本" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原本" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'原本'!$A$1:$R$14</definedName>
@@ -17,11 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0&quot;月&quot;"/>
     <numFmt numFmtId="165" formatCode="0_ "/>
     <numFmt numFmtId="166" formatCode="yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;&quot;付&quot;"/>
     <numFmt numFmtId="167" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="168" formatCode="#,##0_);[Red]▲#,##0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -261,7 +262,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -452,6 +453,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -942,7 +949,7 @@
           <t>株価</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n"/>
+      <c r="B3" s="70" t="n"/>
       <c r="C3" s="18" t="inlineStr">
         <is>
           <t>円</t>
@@ -988,7 +995,7 @@
           <t>1年後予想</t>
         </is>
       </c>
-      <c r="B4" s="28" t="n"/>
+      <c r="B4" s="71" t="n"/>
       <c r="C4" s="18" t="inlineStr">
         <is>
           <t>円</t>
@@ -1030,7 +1037,7 @@
           <t>3年後予想</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
+      <c r="B5" s="70" t="n"/>
       <c r="C5" s="18" t="inlineStr">
         <is>
           <t>円</t>
@@ -1055,7 +1062,7 @@
           <t>5年後予想</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
+      <c r="B6" s="70" t="n"/>
       <c r="C6" s="18" t="inlineStr">
         <is>
           <t>円</t>

</xml_diff>

<commit_message>
Always reserve 2 forecast-year columns in execution table; show percentages to 1 decimal
Execution table now always labels the next 2 fiscal years as "YYYY年予想"
columns (filled from J-Quants if disclosed, blank for manual entry
otherwise), reducing visible actual-year history from 6 to 5 to make
room. Profit-margin/checksum rows and dividend yield display 1 decimal
place instead of 2, with no extra rounding applied in code beyond the
cell's display format.
</commit_message>
<xml_diff>
--- a/templates/company_detail_template.xlsx
+++ b/templates/company_detail_template.xlsx
@@ -17,12 +17,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0&quot;月&quot;"/>
     <numFmt numFmtId="165" formatCode="0_ "/>
     <numFmt numFmtId="166" formatCode="yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;&quot;付&quot;"/>
     <numFmt numFmtId="167" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
     <numFmt numFmtId="168" formatCode="#,##0_);[Red]▲#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -262,7 +263,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -458,6 +459,9 @@
     </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -940,7 +944,7 @@
           <t>配当利回り</t>
         </is>
       </c>
-      <c r="Q2" s="23" t="n"/>
+      <c r="Q2" s="72" t="n"/>
       <c r="R2" s="20" t="n"/>
     </row>
     <row r="3" ht="22.5" customHeight="1" s="54">

</xml_diff>